<commit_message>
add a couple more cpu scenarios expected to work as a baseline
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_cpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_cpu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD6F69B5-F5E4-4AF3-968D-5B74488EB85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B6F627-416C-45C2-8DBA-077AB9B6FE2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -89,7 +89,16 @@
     <t>Use</t>
   </si>
   <si>
-    <t>iloc</t>
+    <t>Multi-CPU - MPI</t>
+  </si>
+  <si>
+    <t>mpi</t>
+  </si>
+  <si>
+    <t>Baseline - 1 CPU</t>
+  </si>
+  <si>
+    <t>serial</t>
   </si>
 </sst>
 </file>
@@ -130,7 +139,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -152,6 +161,12 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -245,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -294,6 +309,9 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -355,12 +373,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:N4" totalsRowShown="0">
-  <autoFilter ref="A1:N4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N4">
-    <sortCondition ref="M1:M4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M7" totalsRowShown="0">
+  <autoFilter ref="A1:M7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M7">
+    <sortCondition ref="M1:M7"/>
   </sortState>
-  <tableColumns count="14">
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="device"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode"/>
@@ -374,7 +392,6 @@
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="total_devices"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="devices_per_node"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Use"/>
-    <tableColumn id="14" xr3:uid="{2E707746-4936-409D-83F6-F0094A930949}" name="iloc"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -668,7 +685,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="14" bestFit="1" customWidth="1"/>
@@ -685,7 +702,7 @@
     <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -725,28 +742,25 @@
       <c r="M1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N1" t="s">
-        <v>18</v>
-      </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D2" s="8">
         <v>1</v>
       </c>
       <c r="E2" s="8">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="F2" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" s="8">
         <v>0</v>
@@ -759,73 +773,67 @@
       </c>
       <c r="J2" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="K2" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="L2" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="M2" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
-      <c r="N2">
-        <v>20</v>
-      </c>
     </row>
-    <row r="3" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D3" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="8">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F3" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3" s="8">
         <v>0</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I3" s="9">
         <v>2</v>
       </c>
       <c r="J3" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="K3" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="L3" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="M3" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
-      <c r="N3">
-        <v>28</v>
-      </c>
     </row>
-    <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>11</v>
       </c>
@@ -836,41 +844,173 @@
         <v>13</v>
       </c>
       <c r="D4" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="8">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="F4" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G4" s="8">
         <v>0</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="9">
+        <v>14</v>
+      </c>
+      <c r="I4" s="17">
         <v>2</v>
       </c>
       <c r="J4" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="K4" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="L4" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="M4" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
-      <c r="N4">
-        <v>29</v>
+    </row>
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8">
+        <v>32</v>
+      </c>
+      <c r="F5" s="8">
+        <v>2</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="9">
+        <v>2</v>
+      </c>
+      <c r="J5" s="10">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
+      </c>
+      <c r="K5" s="10">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>64</v>
+      </c>
+      <c r="L5" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M5" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="8">
+        <v>2</v>
+      </c>
+      <c r="E6" s="8">
+        <v>32</v>
+      </c>
+      <c r="F6" s="8">
+        <v>4</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="9">
+        <v>2</v>
+      </c>
+      <c r="J6" s="10">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
+      </c>
+      <c r="K6" s="10">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>128</v>
+      </c>
+      <c r="L6" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M6" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="8">
+        <v>2</v>
+      </c>
+      <c r="E7" s="8">
+        <v>64</v>
+      </c>
+      <c r="F7" s="8">
+        <v>2</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="9">
+        <v>2</v>
+      </c>
+      <c r="J7" s="10">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
+      </c>
+      <c r="K7" s="10">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>128</v>
+      </c>
+      <c r="L7" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M7" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
run full CPU sensitivity sweep
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_cpu.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_cpu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC84055-C68E-4FD8-838F-15310D5DF545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28E7D7B-D4CB-4E56-8FE6-3DCC53E227AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="17">
   <si>
     <t>run_mode</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>standard</t>
+  </si>
+  <si>
+    <t>parallel</t>
   </si>
   <si>
     <t>mem_gb_per_cpu</t>
@@ -121,7 +124,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -136,6 +139,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -205,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -242,6 +251,9 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -303,10 +315,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K5" totalsRowShown="0">
-  <autoFilter ref="A1:K5" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K5">
-    <sortCondition ref="I1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K21" totalsRowShown="0">
+  <autoFilter ref="A1:K21" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K21">
+    <sortCondition ref="I1:I23"/>
   </sortState>
   <tableColumns count="11">
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode"/>
@@ -613,7 +625,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="11" bestFit="1" customWidth="1"/>
@@ -648,7 +660,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>6</v>
@@ -660,12 +672,12 @@
         <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
@@ -704,7 +716,7 @@
     </row>
     <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="7">
         <v>1</v>
@@ -743,7 +755,7 @@
     </row>
     <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="7">
         <v>1</v>
@@ -780,64 +792,688 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="7">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7">
+        <v>0</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="8">
+        <v>2</v>
+      </c>
+      <c r="H5" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
+      </c>
+      <c r="I5" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>4</v>
+      </c>
+      <c r="J5" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>4</v>
+      </c>
+      <c r="K5" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="7">
+        <v>1</v>
+      </c>
+      <c r="C6" s="7">
+        <v>4</v>
+      </c>
+      <c r="D6" s="7">
+        <v>1</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="8">
+        <v>2</v>
+      </c>
+      <c r="H6" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
+      </c>
+      <c r="I6" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>4</v>
+      </c>
+      <c r="J6" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>4</v>
+      </c>
+      <c r="K6" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="7">
-        <v>1</v>
-      </c>
-      <c r="C5" s="7">
-        <v>2</v>
-      </c>
-      <c r="D5" s="7">
-        <v>2</v>
-      </c>
-      <c r="E5" s="7">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="8">
-        <v>2</v>
-      </c>
-      <c r="H5" s="9">
+      <c r="B7" s="7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="7">
+        <v>2</v>
+      </c>
+      <c r="E7" s="7">
+        <v>0</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="8">
+        <v>2</v>
+      </c>
+      <c r="H7" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I7" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>4</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J7" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>4</v>
       </c>
-      <c r="K5" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6"/>
-      <c r="B6"/>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="H6"/>
-      <c r="I6"/>
-      <c r="J6"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7"/>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="H7"/>
-      <c r="I7"/>
-      <c r="J7"/>
+      <c r="K7" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7">
+        <v>8</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="8">
+        <v>2</v>
+      </c>
+      <c r="H8" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="I8" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="J8" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="K8" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7">
+        <v>8</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7">
+        <v>0</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="8">
+        <v>2</v>
+      </c>
+      <c r="H9" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="I9" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="J9" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="K9" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7">
+        <v>1</v>
+      </c>
+      <c r="C10" s="7">
+        <v>2</v>
+      </c>
+      <c r="D10" s="7">
+        <v>4</v>
+      </c>
+      <c r="E10" s="7">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="8">
+        <v>2</v>
+      </c>
+      <c r="H10" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="I10" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="J10" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="K10" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="7">
+        <v>1</v>
+      </c>
+      <c r="C11" s="7">
+        <v>16</v>
+      </c>
+      <c r="D11" s="7">
+        <v>1</v>
+      </c>
+      <c r="E11" s="7">
+        <v>0</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="8">
+        <v>2</v>
+      </c>
+      <c r="H11" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="I11" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="J11" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="K11" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7">
+        <v>2</v>
+      </c>
+      <c r="D12" s="7">
+        <v>8</v>
+      </c>
+      <c r="E12" s="7">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="13">
+        <v>2</v>
+      </c>
+      <c r="H12" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="I12" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="J12" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="K12" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="7">
+        <v>1</v>
+      </c>
+      <c r="C13" s="7">
+        <v>1</v>
+      </c>
+      <c r="D13" s="7">
+        <v>16</v>
+      </c>
+      <c r="E13" s="7">
+        <v>0</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="8">
+        <v>2</v>
+      </c>
+      <c r="H13" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="I13" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="J13" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="K13" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="7">
+        <v>1</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7">
+        <v>32</v>
+      </c>
+      <c r="E14" s="7">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="8">
+        <v>2</v>
+      </c>
+      <c r="H14" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
+      </c>
+      <c r="I14" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>32</v>
+      </c>
+      <c r="J14" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="K14" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="7">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7">
+        <v>2</v>
+      </c>
+      <c r="D15" s="7">
+        <v>16</v>
+      </c>
+      <c r="E15" s="7">
+        <v>0</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="8">
+        <v>2</v>
+      </c>
+      <c r="H15" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
+      </c>
+      <c r="I15" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>32</v>
+      </c>
+      <c r="J15" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="K15" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="7">
+        <v>1</v>
+      </c>
+      <c r="C16" s="7">
+        <v>32</v>
+      </c>
+      <c r="D16" s="7">
+        <v>2</v>
+      </c>
+      <c r="E16" s="7">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="8">
+        <v>2</v>
+      </c>
+      <c r="H16" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
+      </c>
+      <c r="I16" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>64</v>
+      </c>
+      <c r="J16" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="K16" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7">
+        <v>1</v>
+      </c>
+      <c r="C17" s="7">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7">
+        <v>64</v>
+      </c>
+      <c r="E17" s="7">
+        <v>0</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="8">
+        <v>2</v>
+      </c>
+      <c r="H17" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
+      </c>
+      <c r="I17" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>64</v>
+      </c>
+      <c r="J17" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="K17" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="7">
+        <v>1</v>
+      </c>
+      <c r="C18" s="7">
+        <v>2</v>
+      </c>
+      <c r="D18" s="7">
+        <v>32</v>
+      </c>
+      <c r="E18" s="7">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="8">
+        <v>2</v>
+      </c>
+      <c r="H18" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
+      </c>
+      <c r="I18" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>64</v>
+      </c>
+      <c r="J18" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="K18" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="7">
+        <v>2</v>
+      </c>
+      <c r="C19" s="7">
+        <v>32</v>
+      </c>
+      <c r="D19" s="7">
+        <v>4</v>
+      </c>
+      <c r="E19" s="7">
+        <v>0</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="8">
+        <v>2</v>
+      </c>
+      <c r="H19" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
+      </c>
+      <c r="I19" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>128</v>
+      </c>
+      <c r="J19" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="K19" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="7">
+        <v>2</v>
+      </c>
+      <c r="C20" s="7">
+        <v>64</v>
+      </c>
+      <c r="D20" s="7">
+        <v>2</v>
+      </c>
+      <c r="E20" s="7">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="8">
+        <v>2</v>
+      </c>
+      <c r="H20" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
+      </c>
+      <c r="I20" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>128</v>
+      </c>
+      <c r="J20" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="K20" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="7">
+        <v>1</v>
+      </c>
+      <c r="C21" s="7">
+        <v>2</v>
+      </c>
+      <c r="D21" s="7">
+        <v>64</v>
+      </c>
+      <c r="E21" s="7">
+        <v>0</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" s="8">
+        <v>2</v>
+      </c>
+      <c r="H21" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
+      </c>
+      <c r="I21" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>128</v>
+      </c>
+      <c r="J21" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>128</v>
+      </c>
+      <c r="K21" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22"/>
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="H22"/>
+      <c r="I22"/>
+      <c r="J22"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23"/>
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="H23"/>
+      <c r="I23"/>
+      <c r="J23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>